<commit_message>
Append: 2026-03-20 06:52 JST
</commit_message>
<xml_diff>
--- a/案件情報.xlsx
+++ b/案件情報.xlsx
@@ -424,17 +424,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="51" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -479,773 +479,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-02-18 02:33:59</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>大企業の業務効率化AIプロジェクトの技術方針策定を支援するAIテックリード募集</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>システム開発</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>300,000 円 ~ 500,000 円 / 固定</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>期限情報なし</t>
-        </is>
-      </c>
-      <c r="F2" s="1" t="inlineStr">
-        <is>
-          <t>https://www.lancers.jp/work/detail/5423720</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>385</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>🔥AI,Ai ◆効率化</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-02-18 02:33:59</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>【週5日】法人向け生成AIサービス(RAG・議事録機能)のコア開発を担うリードエンジニア募集</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>システム開発</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>500,000 円 ~ 1,000,000 円 / 固定</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>期限情報なし</t>
-        </is>
-      </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t>https://www.lancers.jp/work/detail/5460267</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>375</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>🔥AI,Ai ◆開発</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-02-18 02:33:59</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>建設・土木業界向け施工機械のAI自動制御・アタッチメント開発を支援してくださるエンジニア募集</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>システム開発</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>200,000 円 ~ 300,000 円 / 固定</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>期限情報なし</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>https://www.lancers.jp/work/detail/5434128</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>368</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>🔥AI,Ai ◆開発</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-02-18 02:33:59</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>企業のMicrosoft Copilot導入・活用支援AIコンサルタント募集(研修講師・メンター)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>システム開発</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>200,000 円 ~ 300,000 円 / 固定</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>期限情報なし</t>
-        </is>
-      </c>
-      <c r="F5" s="1" t="inlineStr">
-        <is>
-          <t>https://www.lancers.jp/work/detail/5434363</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>348</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>🔥AI,Ai ◆コンサル</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-02-18 02:33:59</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>【急募】生成AI案件を回してくれるパートナー募集!</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>システム開発</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>1,000,000 円 ~ 3,000,000 円 / 固定</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>期限情報なし</t>
-        </is>
-      </c>
-      <c r="F6" s="1" t="inlineStr">
-        <is>
-          <t>https://www.lancers.jp/work/detail/5493776</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
-        <v>310</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>🔥AI,Ai</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-02-18 02:33:59</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>【急募】製造業向け「製造副産物」の状態(硬度)判定AIのフィジビリティ検証(画像認識/動画解析)</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>システム開発</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>200,000 円 ~ 300,000 円 / 固定</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>期限情報なし</t>
-        </is>
-      </c>
-      <c r="F7" s="1" t="inlineStr">
-        <is>
-          <t>https://www.lancers.jp/work/detail/5439158</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
-        <v>303</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>🔥AI,Ai</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-02-18 02:33:59</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>※急募:Flutterによる業務アプリの開発(+next.js)</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>システム開発</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>300,000 円 ~ 500,000 円 / 固定</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>期限情報なし</t>
-        </is>
-      </c>
-      <c r="F8" s="1" t="inlineStr">
-        <is>
-          <t>https://www.lancers.jp/work/detail/5493471</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>225</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>🔥Next.js ◆開発 ◇アプリ</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-02-18 02:33:59</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>※急募:Next.jsによる業務アプリの開発(+Flutter)</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>システム開発</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>300,000 円 ~ 500,000 円 / 固定</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>期限情報なし</t>
-        </is>
-      </c>
-      <c r="F9" s="1" t="inlineStr">
-        <is>
-          <t>https://www.lancers.jp/work/detail/5493475</t>
-        </is>
-      </c>
-      <c r="G9" t="n">
-        <v>225</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>🔥Next.js ◆開発 ◇アプリ</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-02-18 02:33:59</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>初回 【買い切り20万円】Shopeeチャット管理・返信Webツール開発(複数国対応)</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>システム開発</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>100,000 円 ~ 200,000 円 / 固定</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>期限情報なし</t>
-        </is>
-      </c>
-      <c r="F10" s="1" t="inlineStr">
-        <is>
-          <t>https://www.lancers.jp/work/detail/5493016</t>
-        </is>
-      </c>
-      <c r="G10" t="n">
-        <v>163</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>◆ツール,開発 ◇管理</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-02-18 02:33:59</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>【Unity/XRエンジニア募集】製造業DX支援!既存システムと連携するXRアプリ開発</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>システム開発</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>200,000 円 ~ 300,000 円 / 固定</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>期限情報なし</t>
-        </is>
-      </c>
-      <c r="F11" s="1" t="inlineStr">
-        <is>
-          <t>https://www.lancers.jp/work/detail/5454210</t>
-        </is>
-      </c>
-      <c r="G11" t="n">
-        <v>108</v>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>◆開発 ◇アプリ</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-02-18 02:33:59</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>【急募】腸もみマッサージセラピスト向け予約アプリ開発</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>システム開発</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>500,000 円 ~ 1,000,000 円 / 固定</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>期限情報なし</t>
-        </is>
-      </c>
-      <c r="F12" s="1" t="inlineStr">
-        <is>
-          <t>https://www.lancers.jp/work/detail/5493827</t>
-        </is>
-      </c>
-      <c r="G12" t="n">
-        <v>100</v>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>◆開発 ◇アプリ</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-02-18 02:33:59</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>【Java/講師/福岡市内】企業向け新入社員研修のJava講師業務(サブ講師)</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>システム開発</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>100,000 円 ~ 200,000 円 / 固定</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>期限情報なし</t>
-        </is>
-      </c>
-      <c r="F13" s="1" t="inlineStr">
-        <is>
-          <t>https://www.lancers.jp/work/detail/5488955</t>
-        </is>
-      </c>
-      <c r="G13" t="n">
-        <v>78</v>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>★Java</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-02-18 02:33:59</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>【エクセル】教育機関向け教材販売・学習管理システムの構築(DB型設計・マトリックス集計)</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>システム開発</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>20,000 円 ~ 50,000 円 / 固定</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>期限情報なし</t>
-        </is>
-      </c>
-      <c r="F14" s="1" t="inlineStr">
-        <is>
-          <t>https://www.lancers.jp/work/detail/5493275</t>
-        </is>
-      </c>
-      <c r="G14" t="n">
-        <v>48</v>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>◇管理</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-02-18 02:33:59</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>WordPressへ実装するスライダーの制作</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>システム開発</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>50,000 円 ~ 100,000 円 / 固定</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>期限情報なし</t>
-        </is>
-      </c>
-      <c r="F15" s="1" t="inlineStr">
-        <is>
-          <t>https://www.lancers.jp/work/detail/5493927</t>
-        </is>
-      </c>
-      <c r="G15" t="n">
-        <v>33</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>○WordPress</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-02-18 02:33:59</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>【急募】よもぎ蒸しサロンのWebサイトエラー解決依頼</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>システム開発</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>20,000 円 ~ 50,000 円 / 固定</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>期限情報なし</t>
-        </is>
-      </c>
-      <c r="F16" s="1" t="inlineStr">
-        <is>
-          <t>https://www.lancers.jp/work/detail/5493140</t>
-        </is>
-      </c>
-      <c r="G16" t="n">
-        <v>33</v>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>◇サイト</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-02-18 02:33:59</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>【急募】PHPバージョンアップ検証のためのテスト環境構築依頼</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>システム開発</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>20,000 円 ~ 50,000 円 / 固定</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>期限情報なし</t>
-        </is>
-      </c>
-      <c r="F17" s="1" t="inlineStr">
-        <is>
-          <t>https://www.lancers.jp/work/detail/5493555</t>
-        </is>
-      </c>
-      <c r="G17" t="n">
-        <v>28</v>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>○PHP</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2026-02-18 02:33:59</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>【設計済み!作業時間~10時間】Stripe(銀行振込)を用いた月額課金システムの構築</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>システム開発</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>20,000 円 ~ 50,000 円 / 固定</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>期限情報なし</t>
-        </is>
-      </c>
-      <c r="F18" s="1" t="inlineStr">
-        <is>
-          <t>https://www.lancers.jp/work/detail/5493650</t>
-        </is>
-      </c>
-      <c r="G18" t="n">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2026-02-18 02:33:59</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>【設計済み!作業時間~10時間】Stripe(銀行振込)を用いた月額課金システムの構築</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>システム開発</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>20,000 円 ~ 50,000 円 / 固定</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>期限情報なし</t>
-        </is>
-      </c>
-      <c r="F19" s="1" t="inlineStr">
-        <is>
-          <t>https://www.lancers.jp/work/detail/5493449</t>
-        </is>
-      </c>
-      <c r="G19" t="n">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2026-02-18 02:33:59</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>初回 【自社HP構築】AWSを活かした最適なドメイン統合構成の設計・実装支援</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>システム開発</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>50,000 円 ~ 100,000 円 / 固定</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>期限情報なし</t>
-        </is>
-      </c>
-      <c r="F20" s="1" t="inlineStr">
-        <is>
-          <t>https://www.lancers.jp/work/detail/5493714</t>
-        </is>
-      </c>
-      <c r="G20" t="n">
-        <v>18</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId19"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>